<commit_message>
Imputación y corrección de errores por stash
</commit_message>
<xml_diff>
--- a/data/Diccionario_TFM_Completo.xlsx
+++ b/data/Diccionario_TFM_Completo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\GitHub\hypertension_management_AI_driven_tool\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38BBC448-641E-4967-BAEA-52CA53FED0B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36736746-4D8B-4774-812D-8D0BEAC80311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="758" uniqueCount="453">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="758" uniqueCount="452">
   <si>
     <t>Bloque</t>
   </si>
@@ -282,9 +282,6 @@
   </si>
   <si>
     <t>BAXPF11</t>
-  </si>
-  <si>
-    <t>1: Pasa, 2: Falla</t>
   </si>
   <si>
     <t>BAXTC11</t>
@@ -2149,7 +2146,7 @@
         <v>13</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E3" s="19" t="s">
         <v>14</v>
@@ -2166,7 +2163,7 @@
         <v>16</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>17</v>
@@ -2186,7 +2183,7 @@
         <v>19</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>20</v>
@@ -2206,7 +2203,7 @@
         <v>22</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>23</v>
@@ -2226,7 +2223,7 @@
         <v>25</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>26</v>
@@ -2246,7 +2243,7 @@
         <v>28</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>29</v>
@@ -2266,10 +2263,10 @@
         <v>31</v>
       </c>
       <c r="C9" s="19" t="s">
+        <v>229</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>230</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>231</v>
       </c>
       <c r="E9" s="19" t="s">
         <v>14</v>
@@ -2286,7 +2283,7 @@
         <v>33</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>34</v>
@@ -2295,7 +2292,7 @@
         <v>14</v>
       </c>
       <c r="F10" s="24" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
@@ -2306,7 +2303,7 @@
         <v>35</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>36</v>
@@ -2326,10 +2323,10 @@
         <v>38</v>
       </c>
       <c r="C12" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="D12" s="9" t="s">
         <v>239</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>240</v>
       </c>
       <c r="E12" s="10" t="s">
         <v>10</v>
@@ -2346,10 +2343,10 @@
         <v>40</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E13" s="19" t="s">
         <v>10</v>
@@ -2366,10 +2363,10 @@
         <v>41</v>
       </c>
       <c r="C14" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="D14" s="3" t="s">
         <v>243</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>244</v>
       </c>
       <c r="E14" s="10" t="s">
         <v>10</v>
@@ -2389,7 +2386,7 @@
         <v>44</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E15" s="19" t="s">
         <v>10</v>
@@ -2406,10 +2403,10 @@
         <v>46</v>
       </c>
       <c r="C16" s="10" t="s">
+        <v>245</v>
+      </c>
+      <c r="D16" s="9" t="s">
         <v>246</v>
-      </c>
-      <c r="D16" s="9" t="s">
-        <v>247</v>
       </c>
       <c r="E16" s="10" t="s">
         <v>10</v>
@@ -2426,10 +2423,10 @@
         <v>49</v>
       </c>
       <c r="C17" s="19" t="s">
+        <v>247</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>248</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>249</v>
       </c>
       <c r="E17" s="19" t="s">
         <v>10</v>
@@ -2446,10 +2443,10 @@
         <v>51</v>
       </c>
       <c r="C18" s="10" t="s">
+        <v>249</v>
+      </c>
+      <c r="D18" s="3" t="s">
         <v>250</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>251</v>
       </c>
       <c r="E18" s="10" t="s">
         <v>10</v>
@@ -2466,10 +2463,10 @@
         <v>53</v>
       </c>
       <c r="C19" s="19" t="s">
+        <v>251</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>252</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>253</v>
       </c>
       <c r="E19" s="19" t="s">
         <v>10</v>
@@ -2486,16 +2483,16 @@
         <v>55</v>
       </c>
       <c r="C20" s="10" t="s">
+        <v>253</v>
+      </c>
+      <c r="D20" s="3" t="s">
         <v>254</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>255</v>
       </c>
       <c r="E20" s="10" t="s">
         <v>14</v>
       </c>
       <c r="F20" s="24" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
@@ -2506,16 +2503,16 @@
         <v>57</v>
       </c>
       <c r="C21" s="19" t="s">
+        <v>255</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>256</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>257</v>
       </c>
       <c r="E21" s="19" t="s">
         <v>14</v>
       </c>
       <c r="F21" s="23" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
@@ -2526,16 +2523,16 @@
         <v>59</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E22" s="10" t="s">
         <v>14</v>
       </c>
       <c r="F22" s="24" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
@@ -2546,10 +2543,10 @@
         <v>61</v>
       </c>
       <c r="C23" s="19" t="s">
+        <v>257</v>
+      </c>
+      <c r="D23" s="2" t="s">
         <v>258</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>259</v>
       </c>
       <c r="E23" s="19" t="s">
         <v>14</v>
@@ -2566,7 +2563,7 @@
         <v>63</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>64</v>
@@ -2586,7 +2583,7 @@
         <v>66</v>
       </c>
       <c r="C25" s="19" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>67</v>
@@ -2606,7 +2603,7 @@
         <v>68</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>69</v>
@@ -2615,7 +2612,7 @@
         <v>14</v>
       </c>
       <c r="F26" s="24" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
@@ -2626,7 +2623,7 @@
         <v>70</v>
       </c>
       <c r="C27" s="19" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>71</v>
@@ -2646,7 +2643,7 @@
         <v>72</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>73</v>
@@ -2655,7 +2652,7 @@
         <v>14</v>
       </c>
       <c r="F28" s="24" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
@@ -2666,7 +2663,7 @@
         <v>74</v>
       </c>
       <c r="C29" s="19" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>75</v>
@@ -2686,7 +2683,7 @@
         <v>76</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>77</v>
@@ -2706,7 +2703,7 @@
         <v>78</v>
       </c>
       <c r="C31" s="19" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>79</v>
@@ -2726,7 +2723,7 @@
         <v>80</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D32" s="3" t="s">
         <v>81</v>
@@ -2746,16 +2743,16 @@
         <v>82</v>
       </c>
       <c r="C33" s="19" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E33" s="19" t="s">
         <v>14</v>
       </c>
       <c r="F33" s="23" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.35">
@@ -2763,19 +2760,19 @@
         <v>58</v>
       </c>
       <c r="B34" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="C34" s="10" t="s">
+        <v>277</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="E34" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F34" s="24" t="s">
         <v>84</v>
-      </c>
-      <c r="C34" s="10" t="s">
-        <v>278</v>
-      </c>
-      <c r="D34" s="3" t="s">
-        <v>282</v>
-      </c>
-      <c r="E34" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="F34" s="24" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
@@ -2783,19 +2780,19 @@
         <v>58</v>
       </c>
       <c r="B35" s="14" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C35" s="19" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E35" s="19" t="s">
         <v>14</v>
       </c>
       <c r="F35" s="23" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.35">
@@ -2803,19 +2800,19 @@
         <v>58</v>
       </c>
       <c r="B36" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E36" s="10" t="s">
         <v>10</v>
       </c>
       <c r="F36" s="24" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
@@ -2823,19 +2820,19 @@
         <v>58</v>
       </c>
       <c r="B37" s="14" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C37" s="19" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="E37" s="19" t="s">
         <v>14</v>
       </c>
       <c r="F37" s="23" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.35">
@@ -2843,19 +2840,19 @@
         <v>58</v>
       </c>
       <c r="B38" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="C38" s="10" t="s">
+        <v>279</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="E38" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F38" s="24" t="s">
         <v>89</v>
-      </c>
-      <c r="C38" s="10" t="s">
-        <v>280</v>
-      </c>
-      <c r="D38" s="3" t="s">
-        <v>282</v>
-      </c>
-      <c r="E38" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="F38" s="24" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
@@ -2863,19 +2860,19 @@
         <v>58</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C39" s="19" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E39" s="19" t="s">
         <v>14</v>
       </c>
       <c r="F39" s="23" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.35">
@@ -2883,430 +2880,430 @@
         <v>58</v>
       </c>
       <c r="B40" s="11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C40" s="10" t="s">
+        <v>280</v>
+      </c>
+      <c r="D40" s="3" t="s">
         <v>281</v>
       </c>
-      <c r="D40" s="3" t="s">
-        <v>282</v>
-      </c>
       <c r="E40" s="10" t="s">
         <v>10</v>
       </c>
       <c r="F40" s="24" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A41" s="28" t="s">
+        <v>92</v>
+      </c>
+      <c r="B41" s="14" t="s">
         <v>93</v>
       </c>
-      <c r="B41" s="14" t="s">
-        <v>94</v>
-      </c>
       <c r="C41" s="19" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E41" s="19" t="s">
         <v>14</v>
       </c>
       <c r="F41" s="23" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A42" s="29" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B42" s="11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E42" s="10" t="s">
         <v>14</v>
       </c>
       <c r="F42" s="24" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A43" s="28" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B43" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="C43" s="19" t="s">
+        <v>286</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="E43" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="F43" s="23" t="s">
         <v>98</v>
-      </c>
-      <c r="C43" s="19" t="s">
-        <v>287</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>293</v>
-      </c>
-      <c r="E43" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="F43" s="23" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" s="29" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B44" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="C44" s="10" t="s">
+        <v>289</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="E44" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F44" s="24" t="s">
         <v>100</v>
-      </c>
-      <c r="C44" s="10" t="s">
-        <v>290</v>
-      </c>
-      <c r="D44" s="3" t="s">
-        <v>296</v>
-      </c>
-      <c r="E44" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="F44" s="24" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A45" s="28" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B45" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="C45" s="19" t="s">
+        <v>287</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="E45" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="F45" s="23" t="s">
         <v>102</v>
-      </c>
-      <c r="C45" s="19" t="s">
-        <v>288</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="E45" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="F45" s="23" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" s="29" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B46" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C46" s="10" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E46" s="10" t="s">
         <v>10</v>
       </c>
       <c r="F46" s="24" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A47" s="28" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B47" s="14" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C47" s="19" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="E47" s="19" t="s">
         <v>10</v>
       </c>
       <c r="F47" s="23" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" s="29" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B48" s="11" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C48" s="10" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="E48" s="10" t="s">
         <v>10</v>
       </c>
       <c r="F48" s="24" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="49" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A49" s="28" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B49" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="C49" s="19" t="s">
+        <v>298</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="E49" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="F49" s="23" t="s">
         <v>107</v>
-      </c>
-      <c r="C49" s="19" t="s">
-        <v>299</v>
-      </c>
-      <c r="D49" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="E49" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="F49" s="23" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" s="29" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B50" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="C50" s="10" t="s">
+        <v>299</v>
+      </c>
+      <c r="D50" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="E50" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F50" s="24" t="s">
         <v>109</v>
-      </c>
-      <c r="C50" s="10" t="s">
-        <v>300</v>
-      </c>
-      <c r="D50" s="3" t="s">
-        <v>303</v>
-      </c>
-      <c r="E50" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="F50" s="24" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A51" s="28" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B51" s="14" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C51" s="19" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="E51" s="19" t="s">
         <v>10</v>
       </c>
       <c r="F51" s="23" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" s="29" t="s">
+        <v>111</v>
+      </c>
+      <c r="B52" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="B52" s="11" t="s">
-        <v>113</v>
-      </c>
       <c r="C52" s="10" t="s">
+        <v>304</v>
+      </c>
+      <c r="D52" s="3" t="s">
         <v>305</v>
-      </c>
-      <c r="D52" s="3" t="s">
-        <v>306</v>
       </c>
       <c r="E52" s="10" t="s">
         <v>14</v>
       </c>
       <c r="F52" s="24" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="53" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A53" s="28" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B53" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="C53" s="19" t="s">
+        <v>307</v>
+      </c>
+      <c r="D53" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="C53" s="19" t="s">
-        <v>308</v>
-      </c>
-      <c r="D53" s="2" t="s">
+      <c r="E53" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="F53" s="23" t="s">
         <v>115</v>
-      </c>
-      <c r="E53" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="F53" s="23" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" s="29" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B54" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="C54" s="10" t="s">
+        <v>308</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="E54" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F54" s="24" t="s">
         <v>117</v>
-      </c>
-      <c r="C54" s="10" t="s">
-        <v>309</v>
-      </c>
-      <c r="D54" s="3" t="s">
-        <v>310</v>
-      </c>
-      <c r="E54" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="F54" s="24" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="55" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A55" s="28" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B55" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="C55" s="19" t="s">
+        <v>311</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="E55" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="F55" s="23" t="s">
         <v>119</v>
-      </c>
-      <c r="C55" s="19" t="s">
-        <v>312</v>
-      </c>
-      <c r="D55" s="2" t="s">
-        <v>311</v>
-      </c>
-      <c r="E55" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="F55" s="23" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="29" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B56" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="C56" s="10" t="s">
+        <v>312</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="E56" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F56" s="24" t="s">
         <v>121</v>
-      </c>
-      <c r="C56" s="10" t="s">
-        <v>313</v>
-      </c>
-      <c r="D56" s="3" t="s">
-        <v>314</v>
-      </c>
-      <c r="E56" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="F56" s="24" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="57" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A57" s="28" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B57" s="14" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C57" s="19" t="s">
+        <v>315</v>
+      </c>
+      <c r="D57" s="2" t="s">
         <v>316</v>
       </c>
-      <c r="D57" s="2" t="s">
-        <v>317</v>
-      </c>
       <c r="E57" s="19" t="s">
         <v>10</v>
       </c>
       <c r="F57" s="23" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" s="29" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B58" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C58" s="10" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>10</v>
       </c>
       <c r="F58" s="24" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="59" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A59" s="28" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B59" s="14" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C59" s="19" t="s">
+        <v>318</v>
+      </c>
+      <c r="D59" s="2" t="s">
         <v>319</v>
       </c>
-      <c r="D59" s="2" t="s">
-        <v>320</v>
-      </c>
       <c r="E59" s="19" t="s">
         <v>10</v>
       </c>
       <c r="F59" s="23" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" s="29" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B60" s="11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C60" s="10" t="s">
+        <v>320</v>
+      </c>
+      <c r="D60" s="3" t="s">
         <v>321</v>
       </c>
-      <c r="D60" s="3" t="s">
-        <v>322</v>
-      </c>
       <c r="E60" s="10" t="s">
         <v>10</v>
       </c>
       <c r="F60" s="24" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="61" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A61" s="28" t="s">
+        <v>126</v>
+      </c>
+      <c r="B61" s="14" t="s">
         <v>127</v>
       </c>
-      <c r="B61" s="14" t="s">
-        <v>128</v>
-      </c>
       <c r="C61" s="19" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="D61" s="2" t="s">
         <v>60</v>
@@ -3315,61 +3312,61 @@
         <v>14</v>
       </c>
       <c r="F61" s="23" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" s="29" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B62" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="C62" s="10" t="s">
+        <v>323</v>
+      </c>
+      <c r="D62" s="3" t="s">
         <v>130</v>
-      </c>
-      <c r="C62" s="10" t="s">
-        <v>324</v>
-      </c>
-      <c r="D62" s="3" t="s">
-        <v>131</v>
       </c>
       <c r="E62" s="10" t="s">
         <v>14</v>
       </c>
       <c r="F62" s="24" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="63" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A63" s="28" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B63" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="C63" s="19" t="s">
+        <v>324</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="E63" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="F63" s="23" t="s">
         <v>133</v>
-      </c>
-      <c r="C63" s="19" t="s">
-        <v>325</v>
-      </c>
-      <c r="D63" s="2" t="s">
-        <v>326</v>
-      </c>
-      <c r="E63" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="F63" s="23" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" s="29" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B64" s="11" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C64" s="10" t="s">
+        <v>326</v>
+      </c>
+      <c r="D64" s="3" t="s">
         <v>327</v>
-      </c>
-      <c r="D64" s="3" t="s">
-        <v>328</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>10</v>
@@ -3380,256 +3377,256 @@
     </row>
     <row r="65" spans="1:6" ht="31" x14ac:dyDescent="0.35">
       <c r="A65" s="28" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B65" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="C65" s="19" t="s">
+        <v>328</v>
+      </c>
+      <c r="D65" s="33" t="s">
+        <v>329</v>
+      </c>
+      <c r="E65" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="F65" s="23" t="s">
         <v>136</v>
-      </c>
-      <c r="C65" s="19" t="s">
-        <v>329</v>
-      </c>
-      <c r="D65" s="33" t="s">
-        <v>330</v>
-      </c>
-      <c r="E65" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="F65" s="23" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" s="29" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B66" s="11" t="s">
+        <v>137</v>
+      </c>
+      <c r="C66" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="D66" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="E66" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F66" s="24" t="s">
         <v>138</v>
-      </c>
-      <c r="C66" s="10" t="s">
-        <v>331</v>
-      </c>
-      <c r="D66" s="3" t="s">
-        <v>332</v>
-      </c>
-      <c r="E66" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="F66" s="24" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="67" spans="1:6" ht="31" x14ac:dyDescent="0.35">
       <c r="A67" s="28" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B67" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="C67" s="19" t="s">
+        <v>332</v>
+      </c>
+      <c r="D67" s="33" t="s">
+        <v>333</v>
+      </c>
+      <c r="E67" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="F67" s="23" t="s">
         <v>140</v>
-      </c>
-      <c r="C67" s="19" t="s">
-        <v>333</v>
-      </c>
-      <c r="D67" s="33" t="s">
-        <v>334</v>
-      </c>
-      <c r="E67" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="F67" s="23" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="68" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A68" s="29" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B68" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="C68" s="10" t="s">
+        <v>334</v>
+      </c>
+      <c r="D68" s="9" t="s">
+        <v>335</v>
+      </c>
+      <c r="E68" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F68" s="24" t="s">
         <v>142</v>
-      </c>
-      <c r="C68" s="10" t="s">
-        <v>335</v>
-      </c>
-      <c r="D68" s="9" t="s">
-        <v>336</v>
-      </c>
-      <c r="E68" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="F68" s="24" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="69" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A69" s="28" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B69" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="C69" s="19" t="s">
+        <v>336</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="E69" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="F69" s="23" t="s">
         <v>144</v>
-      </c>
-      <c r="C69" s="19" t="s">
-        <v>337</v>
-      </c>
-      <c r="D69" s="2" t="s">
-        <v>338</v>
-      </c>
-      <c r="E69" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="F69" s="23" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70" s="29" t="s">
+        <v>145</v>
+      </c>
+      <c r="B70" s="11" t="s">
         <v>146</v>
       </c>
-      <c r="B70" s="11" t="s">
+      <c r="C70" s="10" t="s">
+        <v>338</v>
+      </c>
+      <c r="D70" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="E70" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F70" s="24" t="s">
         <v>147</v>
-      </c>
-      <c r="C70" s="10" t="s">
-        <v>339</v>
-      </c>
-      <c r="D70" s="3" t="s">
-        <v>340</v>
-      </c>
-      <c r="E70" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="F70" s="24" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="71" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A71" s="28" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B71" s="14" t="s">
+        <v>148</v>
+      </c>
+      <c r="C71" s="19" t="s">
+        <v>340</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="E71" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="F71" s="23" t="s">
         <v>149</v>
-      </c>
-      <c r="C71" s="19" t="s">
-        <v>341</v>
-      </c>
-      <c r="D71" s="2" t="s">
-        <v>342</v>
-      </c>
-      <c r="E71" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="F71" s="23" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" s="29" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B72" s="11" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C72" s="10" t="s">
+        <v>342</v>
+      </c>
+      <c r="D72" s="3" t="s">
         <v>343</v>
-      </c>
-      <c r="D72" s="3" t="s">
-        <v>344</v>
       </c>
       <c r="E72" s="10" t="s">
         <v>14</v>
       </c>
       <c r="F72" s="24" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="73" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A73" s="28" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B73" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="C73" s="19" t="s">
+        <v>344</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="E73" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="F73" s="23" t="s">
         <v>153</v>
-      </c>
-      <c r="C73" s="19" t="s">
-        <v>345</v>
-      </c>
-      <c r="D73" s="2" t="s">
-        <v>349</v>
-      </c>
-      <c r="E73" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="F73" s="23" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" s="29" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B74" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="C74" s="10" t="s">
+        <v>345</v>
+      </c>
+      <c r="D74" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="E74" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F74" s="24" t="s">
         <v>155</v>
-      </c>
-      <c r="C74" s="10" t="s">
-        <v>346</v>
-      </c>
-      <c r="D74" s="3" t="s">
-        <v>347</v>
-      </c>
-      <c r="E74" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="F74" s="24" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="75" spans="1:6" ht="31" x14ac:dyDescent="0.35">
       <c r="A75" s="28" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B75" s="14" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C75" s="19" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="D75" s="33" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="E75" s="19" t="s">
         <v>14</v>
       </c>
       <c r="F75" s="23" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76" s="29" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B76" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="C76" s="10" t="s">
+        <v>350</v>
+      </c>
+      <c r="D76" s="3" t="s">
+        <v>351</v>
+      </c>
+      <c r="E76" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F76" s="24" t="s">
         <v>158</v>
-      </c>
-      <c r="C76" s="10" t="s">
-        <v>351</v>
-      </c>
-      <c r="D76" s="3" t="s">
-        <v>352</v>
-      </c>
-      <c r="E76" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="F76" s="24" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="77" spans="1:6" ht="31" x14ac:dyDescent="0.35">
       <c r="A77" s="28" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B77" s="14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C77" s="19" t="s">
+        <v>352</v>
+      </c>
+      <c r="D77" s="33" t="s">
         <v>353</v>
-      </c>
-      <c r="D77" s="33" t="s">
-        <v>354</v>
       </c>
       <c r="E77" s="19" t="s">
         <v>10</v>
@@ -3640,476 +3637,476 @@
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A78" s="29" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B78" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="C78" s="10" t="s">
+        <v>354</v>
+      </c>
+      <c r="D78" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="E78" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F78" s="24" t="s">
         <v>161</v>
-      </c>
-      <c r="C78" s="10" t="s">
-        <v>355</v>
-      </c>
-      <c r="D78" s="3" t="s">
-        <v>356</v>
-      </c>
-      <c r="E78" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="F78" s="24" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="79" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A79" s="28" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B79" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C79" s="19" t="s">
+        <v>356</v>
+      </c>
+      <c r="D79" s="2" t="s">
         <v>357</v>
-      </c>
-      <c r="D79" s="2" t="s">
-        <v>358</v>
       </c>
       <c r="E79" s="19" t="s">
         <v>14</v>
       </c>
       <c r="F79" s="23" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80" s="29" t="s">
+        <v>163</v>
+      </c>
+      <c r="B80" s="11" t="s">
         <v>164</v>
       </c>
-      <c r="B80" s="11" t="s">
+      <c r="C80" s="10" t="s">
+        <v>358</v>
+      </c>
+      <c r="D80" s="3" t="s">
+        <v>359</v>
+      </c>
+      <c r="E80" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F80" s="24" t="s">
         <v>165</v>
-      </c>
-      <c r="C80" s="10" t="s">
-        <v>359</v>
-      </c>
-      <c r="D80" s="3" t="s">
-        <v>360</v>
-      </c>
-      <c r="E80" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="F80" s="24" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="81" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A81" s="28" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B81" s="14" t="s">
+        <v>166</v>
+      </c>
+      <c r="C81" s="19" t="s">
+        <v>360</v>
+      </c>
+      <c r="D81" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="E81" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="F81" s="23" t="s">
         <v>167</v>
-      </c>
-      <c r="C81" s="19" t="s">
-        <v>361</v>
-      </c>
-      <c r="D81" s="2" t="s">
-        <v>362</v>
-      </c>
-      <c r="E81" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="F81" s="23" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A82" s="29" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B82" s="11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C82" s="10" t="s">
+        <v>362</v>
+      </c>
+      <c r="D82" s="3" t="s">
         <v>363</v>
       </c>
-      <c r="D82" s="3" t="s">
-        <v>364</v>
-      </c>
       <c r="E82" s="10" t="s">
         <v>10</v>
       </c>
       <c r="F82" s="24" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="83" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A83" s="28" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B83" s="14" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C83" s="19" t="s">
+        <v>364</v>
+      </c>
+      <c r="D83" s="2" t="s">
         <v>365</v>
       </c>
-      <c r="D83" s="2" t="s">
-        <v>366</v>
-      </c>
       <c r="E83" s="19" t="s">
         <v>10</v>
       </c>
       <c r="F83" s="23" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A84" s="29" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B84" s="11" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C84" s="10" t="s">
+        <v>366</v>
+      </c>
+      <c r="D84" s="3" t="s">
         <v>367</v>
       </c>
-      <c r="D84" s="3" t="s">
-        <v>368</v>
-      </c>
       <c r="E84" s="10" t="s">
         <v>10</v>
       </c>
       <c r="F84" s="24" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="85" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A85" s="28" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B85" s="14" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C85" s="19" t="s">
+        <v>368</v>
+      </c>
+      <c r="D85" s="2" t="s">
         <v>369</v>
       </c>
-      <c r="D85" s="2" t="s">
-        <v>370</v>
-      </c>
       <c r="E85" s="19" t="s">
         <v>10</v>
       </c>
       <c r="F85" s="23" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A86" s="29" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B86" s="11" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C86" s="10" t="s">
+        <v>370</v>
+      </c>
+      <c r="D86" s="9" t="s">
         <v>371</v>
       </c>
-      <c r="D86" s="9" t="s">
-        <v>372</v>
-      </c>
       <c r="E86" s="10" t="s">
         <v>10</v>
       </c>
       <c r="F86" s="24" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="87" spans="1:6" ht="31" x14ac:dyDescent="0.35">
       <c r="A87" s="28" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B87" s="14" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C87" s="19" t="s">
+        <v>372</v>
+      </c>
+      <c r="D87" s="33" t="s">
         <v>373</v>
       </c>
-      <c r="D87" s="33" t="s">
-        <v>374</v>
-      </c>
       <c r="E87" s="19" t="s">
         <v>10</v>
       </c>
       <c r="F87" s="23" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="88" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A88" s="29" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B88" s="11" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C88" s="10" t="s">
+        <v>374</v>
+      </c>
+      <c r="D88" s="9" t="s">
         <v>375</v>
       </c>
-      <c r="D88" s="9" t="s">
-        <v>376</v>
-      </c>
       <c r="E88" s="10" t="s">
         <v>10</v>
       </c>
       <c r="F88" s="24" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="89" spans="1:6" ht="31" x14ac:dyDescent="0.35">
       <c r="A89" s="28" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B89" s="14" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C89" s="19" t="s">
+        <v>376</v>
+      </c>
+      <c r="D89" s="33" t="s">
         <v>377</v>
       </c>
-      <c r="D89" s="33" t="s">
-        <v>378</v>
-      </c>
       <c r="E89" s="19" t="s">
         <v>10</v>
       </c>
       <c r="F89" s="23" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A90" s="29" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B90" s="11" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C90" s="10" t="s">
+        <v>378</v>
+      </c>
+      <c r="D90" s="3" t="s">
         <v>379</v>
       </c>
-      <c r="D90" s="3" t="s">
-        <v>380</v>
-      </c>
       <c r="E90" s="10" t="s">
         <v>10</v>
       </c>
       <c r="F90" s="24" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="91" spans="1:6" ht="31" x14ac:dyDescent="0.35">
       <c r="A91" s="28" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B91" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="C91" s="19" t="s">
+        <v>380</v>
+      </c>
+      <c r="D91" s="33" t="s">
+        <v>381</v>
+      </c>
+      <c r="E91" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="F91" s="23" t="s">
         <v>178</v>
-      </c>
-      <c r="C91" s="19" t="s">
-        <v>381</v>
-      </c>
-      <c r="D91" s="33" t="s">
-        <v>382</v>
-      </c>
-      <c r="E91" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="F91" s="23" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A92" s="29" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B92" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="C92" s="10" t="s">
+        <v>382</v>
+      </c>
+      <c r="D92" s="3" t="s">
+        <v>383</v>
+      </c>
+      <c r="E92" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F92" s="24" t="s">
         <v>180</v>
-      </c>
-      <c r="C92" s="10" t="s">
-        <v>383</v>
-      </c>
-      <c r="D92" s="3" t="s">
-        <v>384</v>
-      </c>
-      <c r="E92" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="F92" s="24" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="93" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A93" s="28" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B93" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C93" s="19" t="s">
+        <v>384</v>
+      </c>
+      <c r="D93" s="2" t="s">
         <v>385</v>
       </c>
-      <c r="D93" s="2" t="s">
-        <v>386</v>
-      </c>
       <c r="E93" s="19" t="s">
         <v>10</v>
       </c>
       <c r="F93" s="23" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A94" s="29" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B94" s="11" t="s">
+        <v>182</v>
+      </c>
+      <c r="C94" s="10" t="s">
+        <v>386</v>
+      </c>
+      <c r="D94" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="E94" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F94" s="24" t="s">
         <v>183</v>
-      </c>
-      <c r="C94" s="10" t="s">
-        <v>387</v>
-      </c>
-      <c r="D94" s="3" t="s">
-        <v>388</v>
-      </c>
-      <c r="E94" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="F94" s="24" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="95" spans="1:6" ht="31" x14ac:dyDescent="0.35">
       <c r="A95" s="28" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B95" s="14" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C95" s="19" t="s">
+        <v>388</v>
+      </c>
+      <c r="D95" s="33" t="s">
         <v>389</v>
       </c>
-      <c r="D95" s="33" t="s">
-        <v>390</v>
-      </c>
       <c r="E95" s="19" t="s">
         <v>10</v>
       </c>
       <c r="F95" s="23" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A96" s="29" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B96" s="11" t="s">
+        <v>185</v>
+      </c>
+      <c r="C96" s="10" t="s">
+        <v>390</v>
+      </c>
+      <c r="D96" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="E96" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F96" s="24" t="s">
         <v>186</v>
-      </c>
-      <c r="C96" s="10" t="s">
-        <v>391</v>
-      </c>
-      <c r="D96" s="3" t="s">
-        <v>392</v>
-      </c>
-      <c r="E96" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="F96" s="24" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="97" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A97" s="28" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B97" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C97" s="19" t="s">
+        <v>392</v>
+      </c>
+      <c r="D97" s="2" t="s">
         <v>393</v>
       </c>
-      <c r="D97" s="2" t="s">
-        <v>394</v>
-      </c>
       <c r="E97" s="19" t="s">
         <v>10</v>
       </c>
       <c r="F97" s="23" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A98" s="29" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B98" s="11" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C98" s="10" t="s">
+        <v>394</v>
+      </c>
+      <c r="D98" s="3" t="s">
         <v>395</v>
       </c>
-      <c r="D98" s="3" t="s">
-        <v>396</v>
-      </c>
       <c r="E98" s="10" t="s">
         <v>10</v>
       </c>
       <c r="F98" s="24" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="99" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A99" s="28" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B99" s="14" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C99" s="19" t="s">
+        <v>396</v>
+      </c>
+      <c r="D99" s="2" t="s">
         <v>397</v>
       </c>
-      <c r="D99" s="2" t="s">
-        <v>398</v>
-      </c>
       <c r="E99" s="19" t="s">
         <v>10</v>
       </c>
       <c r="F99" s="23" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A100" s="29" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B100" s="11" t="s">
+        <v>190</v>
+      </c>
+      <c r="C100" s="10" t="s">
+        <v>398</v>
+      </c>
+      <c r="D100" s="3" t="s">
+        <v>399</v>
+      </c>
+      <c r="E100" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F100" s="24" t="s">
         <v>191</v>
-      </c>
-      <c r="C100" s="10" t="s">
-        <v>399</v>
-      </c>
-      <c r="D100" s="3" t="s">
-        <v>400</v>
-      </c>
-      <c r="E100" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="F100" s="24" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="101" spans="1:6" ht="31" x14ac:dyDescent="0.35">
       <c r="A101" s="28" t="s">
+        <v>192</v>
+      </c>
+      <c r="B101" s="14" t="s">
         <v>193</v>
       </c>
-      <c r="B101" s="14" t="s">
-        <v>194</v>
-      </c>
       <c r="C101" s="19" t="s">
+        <v>400</v>
+      </c>
+      <c r="D101" s="33" t="s">
         <v>401</v>
-      </c>
-      <c r="D101" s="33" t="s">
-        <v>402</v>
       </c>
       <c r="E101" s="19" t="s">
         <v>10</v>
@@ -4120,507 +4117,507 @@
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A102" s="29" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B102" s="11" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C102" s="10" t="s">
+        <v>402</v>
+      </c>
+      <c r="D102" s="3" t="s">
         <v>403</v>
       </c>
-      <c r="D102" s="3" t="s">
-        <v>404</v>
-      </c>
       <c r="E102" s="10" t="s">
         <v>10</v>
       </c>
       <c r="F102" s="24" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="103" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A103" s="28" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B103" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="C103" s="19" t="s">
+        <v>404</v>
+      </c>
+      <c r="D103" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="E103" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="F103" s="23" t="s">
         <v>196</v>
-      </c>
-      <c r="C103" s="19" t="s">
-        <v>405</v>
-      </c>
-      <c r="D103" s="2" t="s">
-        <v>406</v>
-      </c>
-      <c r="E103" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="F103" s="23" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="104" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A104" s="29" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B104" s="11" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C104" s="10" t="s">
+        <v>406</v>
+      </c>
+      <c r="D104" s="9" t="s">
         <v>407</v>
       </c>
-      <c r="D104" s="9" t="s">
-        <v>408</v>
-      </c>
       <c r="E104" s="10" t="s">
         <v>10</v>
       </c>
       <c r="F104" s="24" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="105" spans="1:6" ht="31" x14ac:dyDescent="0.35">
       <c r="A105" s="28" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B105" s="14" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C105" s="19" t="s">
+        <v>408</v>
+      </c>
+      <c r="D105" s="33" t="s">
         <v>409</v>
       </c>
-      <c r="D105" s="33" t="s">
-        <v>410</v>
-      </c>
       <c r="E105" s="19" t="s">
         <v>10</v>
       </c>
       <c r="F105" s="23" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="106" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A106" s="29" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B106" s="11" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C106" s="10" t="s">
+        <v>410</v>
+      </c>
+      <c r="D106" s="9" t="s">
         <v>411</v>
       </c>
-      <c r="D106" s="9" t="s">
-        <v>412</v>
-      </c>
       <c r="E106" s="10" t="s">
         <v>10</v>
       </c>
       <c r="F106" s="24" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="107" spans="1:6" ht="31" x14ac:dyDescent="0.35">
       <c r="A107" s="28" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B107" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C107" s="19" t="s">
+        <v>412</v>
+      </c>
+      <c r="D107" s="33" t="s">
         <v>413</v>
       </c>
-      <c r="D107" s="33" t="s">
-        <v>414</v>
-      </c>
       <c r="E107" s="19" t="s">
         <v>10</v>
       </c>
       <c r="F107" s="23" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A108" s="29" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B108" s="11" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C108" s="10" t="s">
+        <v>414</v>
+      </c>
+      <c r="D108" s="3" t="s">
         <v>415</v>
       </c>
-      <c r="D108" s="3" t="s">
-        <v>416</v>
-      </c>
       <c r="E108" s="10" t="s">
         <v>10</v>
       </c>
       <c r="F108" s="24" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="109" spans="1:6" ht="31" x14ac:dyDescent="0.35">
       <c r="A109" s="28" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B109" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C109" s="19" t="s">
+        <v>416</v>
+      </c>
+      <c r="D109" s="33" t="s">
         <v>417</v>
       </c>
-      <c r="D109" s="33" t="s">
-        <v>418</v>
-      </c>
       <c r="E109" s="19" t="s">
         <v>10</v>
       </c>
       <c r="F109" s="23" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A110" s="29" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B110" s="11" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C110" s="10" t="s">
+        <v>418</v>
+      </c>
+      <c r="D110" s="3" t="s">
         <v>419</v>
       </c>
-      <c r="D110" s="3" t="s">
-        <v>420</v>
-      </c>
       <c r="E110" s="10" t="s">
         <v>10</v>
       </c>
       <c r="F110" s="24" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="111" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A111" s="28" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B111" s="14" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C111" s="19" t="s">
+        <v>420</v>
+      </c>
+      <c r="D111" s="2" t="s">
         <v>421</v>
       </c>
-      <c r="D111" s="2" t="s">
-        <v>422</v>
-      </c>
       <c r="E111" s="19" t="s">
         <v>10</v>
       </c>
       <c r="F111" s="23" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A112" s="29" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B112" s="11" t="s">
+        <v>205</v>
+      </c>
+      <c r="C112" s="10" t="s">
+        <v>422</v>
+      </c>
+      <c r="D112" s="3" t="s">
+        <v>423</v>
+      </c>
+      <c r="E112" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F112" s="24" t="s">
         <v>206</v>
-      </c>
-      <c r="C112" s="10" t="s">
-        <v>423</v>
-      </c>
-      <c r="D112" s="3" t="s">
-        <v>424</v>
-      </c>
-      <c r="E112" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="F112" s="24" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="113" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A113" s="28" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B113" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C113" s="19" t="s">
+        <v>424</v>
+      </c>
+      <c r="D113" s="2" t="s">
         <v>425</v>
       </c>
-      <c r="D113" s="2" t="s">
-        <v>426</v>
-      </c>
       <c r="E113" s="19" t="s">
         <v>10</v>
       </c>
       <c r="F113" s="23" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A114" s="29" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B114" s="11" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C114" s="10" t="s">
+        <v>426</v>
+      </c>
+      <c r="D114" s="3" t="s">
         <v>427</v>
-      </c>
-      <c r="D114" s="3" t="s">
-        <v>428</v>
       </c>
       <c r="E114" s="10" t="s">
         <v>14</v>
       </c>
       <c r="F114" s="24" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="115" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A115" s="28" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B115" s="14" t="s">
+        <v>209</v>
+      </c>
+      <c r="C115" s="19" t="s">
+        <v>428</v>
+      </c>
+      <c r="D115" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="E115" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="F115" s="23" t="s">
         <v>210</v>
-      </c>
-      <c r="C115" s="19" t="s">
-        <v>429</v>
-      </c>
-      <c r="D115" s="2" t="s">
-        <v>430</v>
-      </c>
-      <c r="E115" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="F115" s="23" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A116" s="29" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B116" s="11" t="s">
+        <v>211</v>
+      </c>
+      <c r="C116" s="10" t="s">
+        <v>430</v>
+      </c>
+      <c r="D116" s="3" t="s">
+        <v>431</v>
+      </c>
+      <c r="E116" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F116" s="24" t="s">
         <v>212</v>
-      </c>
-      <c r="C116" s="10" t="s">
-        <v>431</v>
-      </c>
-      <c r="D116" s="3" t="s">
-        <v>432</v>
-      </c>
-      <c r="E116" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="F116" s="24" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="117" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A117" s="28" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B117" s="14" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C117" s="19" t="s">
+        <v>432</v>
+      </c>
+      <c r="D117" s="2" t="s">
         <v>433</v>
-      </c>
-      <c r="D117" s="2" t="s">
-        <v>434</v>
       </c>
       <c r="E117" s="19" t="s">
         <v>14</v>
       </c>
       <c r="F117" s="23" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A118" s="29" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B118" s="11" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C118" s="10" t="s">
+        <v>434</v>
+      </c>
+      <c r="D118" s="3" t="s">
         <v>435</v>
       </c>
-      <c r="D118" s="3" t="s">
-        <v>436</v>
-      </c>
       <c r="E118" s="10" t="s">
         <v>10</v>
       </c>
       <c r="F118" s="24" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="119" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A119" s="28" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B119" s="14" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C119" s="19" t="s">
+        <v>436</v>
+      </c>
+      <c r="D119" s="2" t="s">
         <v>437</v>
       </c>
-      <c r="D119" s="2" t="s">
-        <v>438</v>
-      </c>
       <c r="E119" s="19" t="s">
         <v>10</v>
       </c>
       <c r="F119" s="23" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A120" s="29" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B120" s="11" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C120" s="10" t="s">
+        <v>438</v>
+      </c>
+      <c r="D120" s="3" t="s">
         <v>439</v>
-      </c>
-      <c r="D120" s="3" t="s">
-        <v>440</v>
       </c>
       <c r="E120" s="10" t="s">
         <v>14</v>
       </c>
       <c r="F120" s="24" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="121" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A121" s="28" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B121" s="14" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C121" s="19" t="s">
+        <v>440</v>
+      </c>
+      <c r="D121" s="2" t="s">
         <v>441</v>
       </c>
-      <c r="D121" s="2" t="s">
-        <v>442</v>
-      </c>
       <c r="E121" s="19" t="s">
         <v>10</v>
       </c>
       <c r="F121" s="23" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A122" s="29" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B122" s="11" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C122" s="10" t="s">
+        <v>442</v>
+      </c>
+      <c r="D122" s="3" t="s">
         <v>443</v>
       </c>
-      <c r="D122" s="3" t="s">
-        <v>444</v>
-      </c>
       <c r="E122" s="10" t="s">
         <v>10</v>
       </c>
       <c r="F122" s="24" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="123" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A123" s="28" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B123" s="14" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C123" s="19" t="s">
+        <v>444</v>
+      </c>
+      <c r="D123" s="2" t="s">
         <v>445</v>
-      </c>
-      <c r="D123" s="2" t="s">
-        <v>446</v>
       </c>
       <c r="E123" s="19" t="s">
         <v>14</v>
       </c>
       <c r="F123" s="23" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A124" s="29" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B124" s="11" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C124" s="10" t="s">
+        <v>446</v>
+      </c>
+      <c r="D124" s="3" t="s">
         <v>447</v>
       </c>
-      <c r="D124" s="3" t="s">
-        <v>448</v>
-      </c>
       <c r="E124" s="10" t="s">
         <v>10</v>
       </c>
       <c r="F124" s="24" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="125" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A125" s="28" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B125" s="14" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C125" s="19" t="s">
+        <v>448</v>
+      </c>
+      <c r="D125" s="2" t="s">
         <v>449</v>
       </c>
-      <c r="D125" s="2" t="s">
-        <v>450</v>
-      </c>
       <c r="E125" s="19" t="s">
         <v>10</v>
       </c>
       <c r="F125" s="23" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="126" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A126" s="30" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B126" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C126" s="20" t="s">
+        <v>450</v>
+      </c>
+      <c r="D126" s="4" t="s">
         <v>451</v>
-      </c>
-      <c r="D126" s="4" t="s">
-        <v>452</v>
       </c>
       <c r="E126" s="20" t="s">
         <v>14</v>
       </c>
       <c r="F126" s="25" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="127" spans="1:6" ht="23.5" x14ac:dyDescent="0.35">
       <c r="A127" s="31" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B127" s="7">
         <f>COUNTIF(E:E,E97)</f>
@@ -4629,7 +4626,7 @@
     </row>
     <row r="128" spans="1:6" ht="24" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A128" s="32" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B128" s="6">
         <f>COUNTIF(E:E,E3)</f>

</xml_diff>